<commit_message>
A complete analysis of all data was conducted and a statistical bar chart was created. --Yunlong Wang,Computing Science,Griffith College Dublin-- 2026/7/11 18:10
</commit_message>
<xml_diff>
--- a/datasets/processed/integral data.xlsx
+++ b/datasets/processed/integral data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wj863\WebstormProjects\Network-Performance-Research\datasets\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BD8203-3BF7-4985-91D3-46C13E190398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3E1272-C7D2-42A3-8BF6-389C471C8AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D220BB92-DB5D-433E-A582-99A154683DFA}"/>
+    <workbookView xWindow="12096" yWindow="1596" windowWidth="12360" windowHeight="10104" xr2:uid="{D220BB92-DB5D-433E-A582-99A154683DFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>